<commit_message>
Addresses natural gas transmission mapping issue
</commit_message>
<xml_diff>
--- a/InputData/bldgs/SoBCaICbIC/Shr of Bldg Cap and Instl Costs by ISIC Code.xlsx
+++ b/InputData/bldgs/SoBCaICbIC/Shr of Bldg Cap and Instl Costs by ISIC Code.xlsx
@@ -35466,7 +35466,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -35474,7 +35474,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="11">
@@ -35499,7 +35499,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -35507,7 +35507,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="12">
@@ -35532,7 +35532,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -35540,7 +35540,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="13">
@@ -35565,7 +35565,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -35573,7 +35573,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="14">
@@ -35598,7 +35598,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -35606,7 +35606,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="15">
@@ -35994,7 +35994,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -36002,7 +36002,7 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="27">
@@ -36027,7 +36027,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -36035,7 +36035,7 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="28">
@@ -36060,7 +36060,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -36068,7 +36068,7 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="29">
@@ -36093,7 +36093,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -36101,7 +36101,7 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="30">
@@ -36126,7 +36126,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -36134,7 +36134,7 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="31">
@@ -36522,7 +36522,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -36530,7 +36530,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="43">
@@ -36555,7 +36555,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -36563,7 +36563,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="44">
@@ -36588,7 +36588,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -36596,7 +36596,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="45">
@@ -36621,7 +36621,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -36629,7 +36629,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="46">
@@ -36654,7 +36654,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -36662,7 +36662,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="47">
@@ -37050,7 +37050,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -37058,7 +37058,7 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="59">
@@ -37083,7 +37083,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -37091,7 +37091,7 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="60">
@@ -37116,7 +37116,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -37124,7 +37124,7 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="61">
@@ -37149,7 +37149,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -37157,7 +37157,7 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="62">
@@ -37182,7 +37182,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -37190,7 +37190,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="63">
@@ -37578,7 +37578,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -37586,7 +37586,7 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="75">
@@ -37611,7 +37611,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -37619,7 +37619,7 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="76">
@@ -37644,7 +37644,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -37652,7 +37652,7 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="77">
@@ -37677,7 +37677,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -37685,7 +37685,7 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="78">
@@ -37710,7 +37710,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -37718,7 +37718,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="79">
@@ -38106,7 +38106,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -38114,7 +38114,7 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="91">
@@ -38139,7 +38139,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -38147,7 +38147,7 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="92">
@@ -38172,7 +38172,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -38180,7 +38180,7 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="93">
@@ -38205,7 +38205,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -38213,7 +38213,7 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="94">
@@ -38238,7 +38238,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -38246,7 +38246,7 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="95">
@@ -38634,7 +38634,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -38642,7 +38642,7 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="107">
@@ -38667,7 +38667,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -38675,7 +38675,7 @@
         </is>
       </c>
       <c r="G107" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="108">
@@ -38700,7 +38700,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -38708,7 +38708,7 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="109">
@@ -38733,7 +38733,7 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -38741,7 +38741,7 @@
         </is>
       </c>
       <c r="G109" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="110">
@@ -38766,7 +38766,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -38774,7 +38774,7 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="111">
@@ -39162,7 +39162,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -39170,7 +39170,7 @@
         </is>
       </c>
       <c r="G122" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="123">
@@ -39195,7 +39195,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -39203,7 +39203,7 @@
         </is>
       </c>
       <c r="G123" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="124">
@@ -39228,7 +39228,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -39236,7 +39236,7 @@
         </is>
       </c>
       <c r="G124" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="125">
@@ -39261,7 +39261,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -39269,7 +39269,7 @@
         </is>
       </c>
       <c r="G125" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="126">
@@ -39294,7 +39294,7 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -39302,7 +39302,7 @@
         </is>
       </c>
       <c r="G126" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="127">
@@ -39690,7 +39690,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -39698,7 +39698,7 @@
         </is>
       </c>
       <c r="G138" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="139">
@@ -39723,7 +39723,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -39731,7 +39731,7 @@
         </is>
       </c>
       <c r="G139" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="140">
@@ -39756,7 +39756,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -39764,7 +39764,7 @@
         </is>
       </c>
       <c r="G140" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="141">
@@ -39789,7 +39789,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
@@ -39797,7 +39797,7 @@
         </is>
       </c>
       <c r="G141" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="142">
@@ -39822,7 +39822,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -39830,7 +39830,7 @@
         </is>
       </c>
       <c r="G142" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="143">
@@ -40218,7 +40218,7 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
@@ -40226,7 +40226,7 @@
         </is>
       </c>
       <c r="G154" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="155">
@@ -40251,7 +40251,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -40259,7 +40259,7 @@
         </is>
       </c>
       <c r="G155" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="156">
@@ -40284,7 +40284,7 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
@@ -40292,7 +40292,7 @@
         </is>
       </c>
       <c r="G156" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="157">
@@ -40317,7 +40317,7 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
@@ -40325,7 +40325,7 @@
         </is>
       </c>
       <c r="G157" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="158">
@@ -40350,7 +40350,7 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
@@ -40358,7 +40358,7 @@
         </is>
       </c>
       <c r="G158" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="159">
@@ -40746,7 +40746,7 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F170" t="inlineStr">
         <is>
@@ -40754,7 +40754,7 @@
         </is>
       </c>
       <c r="G170" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="171">
@@ -40779,7 +40779,7 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F171" t="inlineStr">
         <is>
@@ -40787,7 +40787,7 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="172">
@@ -40812,7 +40812,7 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F172" t="inlineStr">
         <is>
@@ -40820,7 +40820,7 @@
         </is>
       </c>
       <c r="G172" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="173">
@@ -40845,7 +40845,7 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F173" t="inlineStr">
         <is>
@@ -40853,7 +40853,7 @@
         </is>
       </c>
       <c r="G173" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="174">
@@ -40878,7 +40878,7 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
@@ -40886,7 +40886,7 @@
         </is>
       </c>
       <c r="G174" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="175">
@@ -41274,7 +41274,7 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F186" t="inlineStr">
         <is>
@@ -41282,7 +41282,7 @@
         </is>
       </c>
       <c r="G186" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="187">
@@ -41307,7 +41307,7 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
@@ -41315,7 +41315,7 @@
         </is>
       </c>
       <c r="G187" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="188">
@@ -41340,7 +41340,7 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F188" t="inlineStr">
         <is>
@@ -41348,7 +41348,7 @@
         </is>
       </c>
       <c r="G188" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="189">
@@ -41373,7 +41373,7 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F189" t="inlineStr">
         <is>
@@ -41381,7 +41381,7 @@
         </is>
       </c>
       <c r="G189" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="190">
@@ -41406,7 +41406,7 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F190" t="inlineStr">
         <is>
@@ -41414,7 +41414,7 @@
         </is>
       </c>
       <c r="G190" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="191">
@@ -41802,7 +41802,7 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F202" t="inlineStr">
         <is>
@@ -41810,7 +41810,7 @@
         </is>
       </c>
       <c r="G202" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="203">
@@ -41835,7 +41835,7 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F203" t="inlineStr">
         <is>
@@ -41843,7 +41843,7 @@
         </is>
       </c>
       <c r="G203" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="204">
@@ -41868,7 +41868,7 @@
         </is>
       </c>
       <c r="E204" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F204" t="inlineStr">
         <is>
@@ -41876,7 +41876,7 @@
         </is>
       </c>
       <c r="G204" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="205">
@@ -41901,7 +41901,7 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F205" t="inlineStr">
         <is>
@@ -41909,7 +41909,7 @@
         </is>
       </c>
       <c r="G205" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="206">
@@ -41934,7 +41934,7 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F206" t="inlineStr">
         <is>
@@ -41942,7 +41942,7 @@
         </is>
       </c>
       <c r="G206" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="207">
@@ -42330,7 +42330,7 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F218" t="inlineStr">
         <is>
@@ -42338,7 +42338,7 @@
         </is>
       </c>
       <c r="G218" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="219">
@@ -42363,7 +42363,7 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F219" t="inlineStr">
         <is>
@@ -42371,7 +42371,7 @@
         </is>
       </c>
       <c r="G219" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="220">
@@ -42396,7 +42396,7 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F220" t="inlineStr">
         <is>
@@ -42404,7 +42404,7 @@
         </is>
       </c>
       <c r="G220" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="221">
@@ -42429,7 +42429,7 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F221" t="inlineStr">
         <is>
@@ -42437,7 +42437,7 @@
         </is>
       </c>
       <c r="G221" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="222">
@@ -42462,7 +42462,7 @@
         </is>
       </c>
       <c r="E222" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F222" t="inlineStr">
         <is>
@@ -42470,7 +42470,7 @@
         </is>
       </c>
       <c r="G222" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="223">
@@ -42858,7 +42858,7 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F234" t="inlineStr">
         <is>
@@ -42866,7 +42866,7 @@
         </is>
       </c>
       <c r="G234" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="235">
@@ -42891,7 +42891,7 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F235" t="inlineStr">
         <is>
@@ -42899,7 +42899,7 @@
         </is>
       </c>
       <c r="G235" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="236">
@@ -42924,7 +42924,7 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F236" t="inlineStr">
         <is>
@@ -42932,7 +42932,7 @@
         </is>
       </c>
       <c r="G236" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="237">
@@ -42957,7 +42957,7 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F237" t="inlineStr">
         <is>
@@ -42965,7 +42965,7 @@
         </is>
       </c>
       <c r="G237" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="238">
@@ -42990,7 +42990,7 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F238" t="inlineStr">
         <is>
@@ -42998,7 +42998,7 @@
         </is>
       </c>
       <c r="G238" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="239">
@@ -43386,7 +43386,7 @@
         </is>
       </c>
       <c r="E250" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F250" t="inlineStr">
         <is>
@@ -43394,7 +43394,7 @@
         </is>
       </c>
       <c r="G250" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="251">
@@ -43419,7 +43419,7 @@
         </is>
       </c>
       <c r="E251" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F251" t="inlineStr">
         <is>
@@ -43427,7 +43427,7 @@
         </is>
       </c>
       <c r="G251" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="252">
@@ -43452,7 +43452,7 @@
         </is>
       </c>
       <c r="E252" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F252" t="inlineStr">
         <is>
@@ -43460,7 +43460,7 @@
         </is>
       </c>
       <c r="G252" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="253">
@@ -43485,7 +43485,7 @@
         </is>
       </c>
       <c r="E253" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F253" t="inlineStr">
         <is>
@@ -43493,7 +43493,7 @@
         </is>
       </c>
       <c r="G253" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="254">
@@ -43518,7 +43518,7 @@
         </is>
       </c>
       <c r="E254" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F254" t="inlineStr">
         <is>
@@ -43526,7 +43526,7 @@
         </is>
       </c>
       <c r="G254" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="255">
@@ -43914,7 +43914,7 @@
         </is>
       </c>
       <c r="E266" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F266" t="inlineStr">
         <is>
@@ -43922,7 +43922,7 @@
         </is>
       </c>
       <c r="G266" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="267">
@@ -43947,7 +43947,7 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F267" t="inlineStr">
         <is>
@@ -43955,7 +43955,7 @@
         </is>
       </c>
       <c r="G267" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="268">
@@ -43980,7 +43980,7 @@
         </is>
       </c>
       <c r="E268" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F268" t="inlineStr">
         <is>
@@ -43988,7 +43988,7 @@
         </is>
       </c>
       <c r="G268" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="269">
@@ -44013,7 +44013,7 @@
         </is>
       </c>
       <c r="E269" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F269" t="inlineStr">
         <is>
@@ -44021,7 +44021,7 @@
         </is>
       </c>
       <c r="G269" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="270">
@@ -44046,7 +44046,7 @@
         </is>
       </c>
       <c r="E270" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F270" t="inlineStr">
         <is>
@@ -44054,7 +44054,7 @@
         </is>
       </c>
       <c r="G270" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="271">
@@ -44442,7 +44442,7 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
       <c r="F282" t="inlineStr">
         <is>
@@ -44450,7 +44450,7 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>0.4781643011829615</v>
+        <v>0.45630816353267</v>
       </c>
     </row>
     <row r="283">
@@ -44475,7 +44475,7 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
       <c r="F283" t="inlineStr">
         <is>
@@ -44483,7 +44483,7 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>0.04258639396614965</v>
+        <v>0.04437004750051631</v>
       </c>
     </row>
     <row r="284">
@@ -44508,7 +44508,7 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
       <c r="F284" t="inlineStr">
         <is>
@@ -44516,7 +44516,7 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>0.1808024634415262</v>
+        <v>0.1883750452665103</v>
       </c>
     </row>
     <row r="285">
@@ -44541,7 +44541,7 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
       <c r="F285" t="inlineStr">
         <is>
@@ -44549,7 +44549,7 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>0.2139060571318126</v>
+        <v>0.2228651226758185</v>
       </c>
     </row>
     <row r="286">
@@ -44574,7 +44574,7 @@
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
       <c r="F286" t="inlineStr">
         <is>
@@ -44582,7 +44582,7 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>0.08454078427755009</v>
+        <v>0.08808162102448482</v>
       </c>
     </row>
     <row r="287">

</xml_diff>